<commit_message>
fix: keep Add project when filter empty; bound task deadline to project dates
Show Add via notFoundContent when no catalog match, clamp/disable deadline outside project start–end, drop create-task project help text, and document TASK-82.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/task-flow-test-cases.xlsx
+++ b/docs/task-flow-test-cases.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Admin: gõ tên project chưa có → Add mở Create project → tạo xong gắn tên + PM (link xanh khi tạo task)</t>
+          <t>Admin: gõ tên project chưa có → Add mở Create project (Add vẫn hiện khi không còn option khớp filter)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1094,32 +1094,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2. Giao task</t>
+          <t>1. Tạo task</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>TASK-06</t>
+          <t>TASK-82</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>PM/Admin tạo task Creative (chưa chọn Staff) → task vào hàng chờ Creative Head</t>
+          <t>Create task: Deadline chỉ chọn ngày trong startDate–endDate của project catalog</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>TASK-47</t>
+          <t>TASK-06</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CH (hoặc Admin/PM) giao task đang ở hàng chờ Creative Head cho một CM → task vào hàng chờ Creative Manager</t>
+          <t>PM/Admin tạo task Creative (chưa chọn Staff) → task vào hàng chờ Creative Head</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1149,9 +1149,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1173,12 +1173,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>TASK-48</t>
+          <t>TASK-47</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Chỉ CH/PM/Admin được chọn CM để giao task; Staff hoặc CM tự giao CM thì bị từ chối (API 403)</t>
+          <t>CH (hoặc Admin/PM) giao task đang ở hàng chờ Creative Head cho một CM → task vào hàng chờ Creative Manager</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1191,9 +1191,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1210,12 +1210,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>TASK-49</t>
+          <t>TASK-48</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Không giao được CM nếu người chọn không phải role CM, hoặc task chưa ở hàng chờ Creative Head (API 422)</t>
+          <t>Chỉ CH/PM/Admin được chọn CM để giao task; Staff hoặc CM tự giao CM thì bị từ chối (API 403)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1247,12 +1247,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>TASK-37</t>
+          <t>TASK-49</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Admin/PM giao (hoặc đổi) Staff trên task phòng Dự án — tối đa 1 người</t>
+          <t>Không giao được CM nếu người chọn không phải role CM, hoặc task chưa ở hàng chờ Creative Head (API 422)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>TASK-50</t>
+          <t>TASK-37</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>CM được giao task đó giao cả khối cho đúng 1 Staff (kèm số lượng)</t>
+          <t>Admin/PM giao (hoặc đổi) Staff trên task phòng Dự án — tối đa 1 người</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1302,9 +1302,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1321,12 +1321,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>TASK-51</t>
+          <t>TASK-50</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>CM chia task thành ≥2 task nhỏ, mỗi phần một Staff + số lượng + brief</t>
+          <t>CM được giao task đó giao cả khối cho đúng 1 Staff (kèm số lượng)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>TASK-52</t>
+          <t>TASK-51</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Chỉ CM đang phụ trách task (hoặc Admin/PM) được giao Staff; Staff thường / CM khác bị 403</t>
+          <t>CM chia task thành ≥2 task nhỏ, mỗi phần một Staff + số lượng + brief</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1376,9 +1376,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1395,12 +1395,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>TASK-58</t>
+          <t>TASK-52</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Giao Staff bị từ chối nếu thiếu Staff, thiếu số lượng, hoặc mode split không đủ task nhỏ hợp lệ</t>
+          <t>Chỉ CM đang phụ trách task (hoặc Admin/PM) được giao Staff; Staff thường / CM khác bị 403</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1432,12 +1432,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>TASK-38</t>
+          <t>TASK-58</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Không cho tạo/giao nếu người nhận đang On leave → 422 `ASSIGNEE_ON_LEAVE` (chặn, không chỉ cảnh báo)</t>
+          <t>Giao Staff bị từ chối nếu thiếu Staff, thiếu số lượng, hoặc mode split không đủ task nhỏ hợp lệ</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1445,14 +1445,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TASK-57</t>
+          <t>TASK-38</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Happy path Creative: tạo → CH giao CM → CM giao Staff (cả khối) thành công</t>
+          <t>Không cho tạo/giao nếu người nhận đang On leave → 422 `ASSIGNEE_ON_LEAVE` (chặn, không chỉ cảnh báo)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1482,14 +1482,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>TASK-55</t>
+          <t>TASK-57</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Khi task còn ở hàng chờ Creative Manager: CH/Admin đổi sang CM khác được; CM không được tự đổi CM</t>
+          <t>Happy path Creative: tạo → CH giao CM → CM giao Staff (cả khối) thành công</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>TASK-59</t>
+          <t>TASK-55</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Sau khi đã giao Staff: CM/Admin (và PM đủ điều kiện) đổi sang Staff khác được</t>
+          <t>Khi task còn ở hàng chờ Creative Manager: CH/Admin đổi sang CM khác được; CM không được tự đổi CM</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1580,12 +1580,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>TASK-60</t>
+          <t>TASK-59</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Task nhỏ Staff đã Confirm: vẫn đổi được số lượng hoặc đổi Staff; đổi Staff thì Confirm về «chưa cập nhật» (Staff Confirm lại). Đã Hoàn thành thì khoá số lượng</t>
+          <t>Sau khi đã giao Staff: CM/Admin (và PM đủ điều kiện) đổi sang Staff khác được</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1593,14 +1593,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>TASK-65</t>
+          <t>TASK-60</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Sau khi CH từ chối task giao: chỉ PM/Admin đưa task lại hàng chờ Creative Head; CH không tự đưa lại</t>
+          <t>Task nhỏ Staff đã Confirm: vẫn đổi được số lượng hoặc đổi Staff; đổi Staff thì Confirm về «chưa cập nhật» (Staff Confirm lại). Đã Hoàn thành thì khoá số lượng</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1630,9 +1630,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1640,9 +1640,9 @@
           <t>~</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>TASK-70</t>
+          <t>TASK-65</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>PM/Admin sửa Deadline PM trên task Creative sau giao Staff được; Staff bị chặn</t>
+          <t>Sau khi CH từ chối task giao: chỉ PM/Admin đưa task lại hàng chờ Creative Head; CH không tự đưa lại</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>TASK-71</t>
+          <t>TASK-70</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Sau giao Staff: CM/PM được sửa Deadline Creative; Creative Head không được sửa field này (API từ chối)</t>
+          <t>PM/Admin sửa Deadline PM trên task Creative sau giao Staff được; Staff bị chặn</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1709,9 +1709,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1728,17 +1728,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>TASK-69</t>
+          <t>TASK-71</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Chỉ CM thấy nút «Task nhận» / «Task giao Staff»; PM, CH, Staff không thấy toggle</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+          <t>Sau giao Staff: CM/PM được sửa Deadline Creative; Creative Head không được sửa field này (API từ chối)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>TASK-69b</t>
+          <t>TASK-69</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Sau chia nhỏ: task cha hiện ở «Task nhận»; từng task con hiện ở «Task giao Staff» (đúng mã/tên)</t>
+          <t>Chỉ CM thấy nút «Task nhận» / «Task giao Staff»; PM, CH, Staff không thấy toggle</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1802,17 +1802,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>TASK-56</t>
+          <t>TASK-69b</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Project Tasks: Admin/PM/CH thấy task cha đã chia, không thấy task con trên list chung; CM xem task con ở tab «Task giao Staff»</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+          <t>Sau chia nhỏ: task cha hiện ở «Task nhận»; từng task con hiện ở «Task giao Staff» (đúng mã/tên)</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1820,14 +1820,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>TASK-35</t>
+          <t>TASK-56</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PM/Admin (có EVALUATE) lưu điểm + % + note trên task</t>
+          <t>Project Tasks: Admin/PM/CH thấy task cha đã chia, không thấy task con trên list chung; CM xem task con ở tab «Task giao Staff»</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1852,9 +1852,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1876,12 +1876,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>TASK-36</t>
+          <t>TASK-35</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Staff không có EVALUATE → không thấy nút Evaluate / API 403</t>
+          <t>PM/Admin (có EVALUATE) lưu điểm + % + note trên task</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>TASK-72</t>
+          <t>TASK-36</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>CH được đánh giá task cha sau khi đã giao CM; CM không được đánh giá task đang ở hàng chờ Creative Manager (chưa giao Staff)</t>
+          <t>Staff không có EVALUATE → không thấy nút Evaluate / API 403</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1926,19 +1926,19 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>~</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -1950,12 +1950,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>TASK-73</t>
+          <t>TASK-72</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>CM đánh giá task đã giao Staff (cả khối / task nhỏ); không đánh giá task cha đã chia nhỏ</t>
+          <t>CH được đánh giá task cha sau khi đã giao CM; CM không được đánh giá task đang ở hàng chờ Creative Manager (chưa giao Staff)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1987,32 +1987,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>TASK-66</t>
+          <t>TASK-73</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>CM đánh giá task nhỏ mà nhận SL thấp hơn đã giao → hệ thống tạo task nhỏ mới cho phần còn lại. Task nhỏ đã Confirm vẫn sửa SL được; đã Hoàn thành thì khoá SL</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
+          <t>CM đánh giá task đã giao Staff (cả khối / task nhỏ); không đánh giá task cha đã chia nhỏ</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>~</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
         </is>
       </c>
     </row>
@@ -2024,17 +2024,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>TASK-74</t>
+          <t>TASK-66</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Sau khi CH đã đánh giá: CM mở task nhận → tab Evaluation thấy điểm/note của CH</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+          <t>CM đánh giá task nhỏ mà nhận SL thấp hơn đã giao → hệ thống tạo task nhỏ mới cho phần còn lại. Task nhỏ đã Confirm vẫn sửa SL được; đã Hoàn thành thì khoá SL</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2042,9 +2042,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>TASK-75</t>
+          <t>TASK-74</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sau khi CM đã đánh giá: Staff mở task mình → tab Evaluation thấy điểm/note của CM</t>
+          <t>Sau khi CH đã đánh giá: CM mở task nhận → tab Evaluation thấy điểm/note của CH</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2098,12 +2098,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>TASK-76</t>
+          <t>TASK-75</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>PM đánh giá task Creative bằng nút Evaluate trên chi tiết task; CM và CH xem điểm/%/note trên tab Evaluation của cùng task (không có màn đánh giá PM riêng)</t>
+          <t>Sau khi CM đã đánh giá: Staff mở task mình → tab Evaluation thấy điểm/note của CM</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -2130,17 +2130,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>3. Từ chối giao</t>
+          <t>2. Giao task</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>TASK-64</t>
+          <t>TASK-76</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Creative Head từ chối nhận task từ PM → task về chờ PM xử lý</t>
+          <t>PM đánh giá task Creative bằng nút Evaluate trên chi tiết task; CM và CH xem điểm/%/note trên tab Evaluation của cùng task (không có màn đánh giá PM riêng)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -2153,14 +2153,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -2172,12 +2172,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>TASK-77</t>
+          <t>TASK-64</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager từ chối nhận → task về hàng chờ Creative Head</t>
+          <t>Creative Head từ chối nhận task từ PM → task về chờ PM xử lý</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -2195,9 +2195,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -2209,12 +2209,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>TASK-78</t>
+          <t>TASK-77</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Staff từ chối task đã giao → task về Creative Manager để giao lại</t>
+          <t>Creative Manager từ chối nhận → task về hàng chờ Creative Head</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -2246,17 +2246,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>TASK-67</t>
+          <t>TASK-78</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Nhập lý do từ chối; lịch sử / tracker ghi nhận đúng</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+          <t>Staff từ chối task đã giao → task về Creative Manager để giao lại</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2264,14 +2264,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
     </row>
@@ -2283,27 +2283,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>TASK-79</t>
+          <t>TASK-67</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Không cho từ chối trên task cha đã chia nhỏ</t>
+          <t>Nhập lý do từ chối; lịch sử / tracker ghi nhận đúng</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2315,37 +2315,37 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>4. Sửa task</t>
+          <t>3. Từ chối giao</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>TASK-07–09</t>
+          <t>TASK-79</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Admin / Head / người tạo được sửa thông tin task</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
+          <t>Không cho từ chối trên task cha đã chia nhỏ</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -2357,12 +2357,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>TASK-10–11</t>
+          <t>TASK-07–09</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>PM không phải người tạo / nhân viên không được sửa meta</t>
+          <t>Admin / Head / người tạo được sửa thông tin task</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2375,9 +2375,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>TASK-12–13</t>
+          <t>TASK-10–11</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Task Hoàn thành / Hủy: không ghi được; vẫn mở xem được</t>
+          <t>PM không phải người tạo / nhân viên không được sửa meta</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2407,9 +2407,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2431,12 +2431,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>TASK-43</t>
+          <t>TASK-12–13</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Đổi mức độ ưu tiên (urgency)</t>
+          <t>Task Hoàn thành / Hủy: không ghi được; vẫn mở xem được</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -2444,14 +2444,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>~</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -2468,12 +2468,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>TASK-53–54</t>
+          <t>TASK-43</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Số lượng trước / sau khi chia nhỏ</t>
+          <t>Đổi mức độ ưu tiên (urgency)</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2505,12 +2505,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>TASK-68</t>
+          <t>TASK-53–54</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Staff mở task cha đã chia nhỏ → không có quyền; PM mở Sửa task đã xong → chỉ xem</t>
+          <t>Số lượng trước / sau khi chia nhỏ</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -2518,36 +2518,36 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>5. Xoá task</t>
+          <t>4. Sửa task</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>TASK-18</t>
+          <t>TASK-68</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Xoá mềm task</t>
+          <t>Staff mở task cha đã chia nhỏ → không có quyền; PM mở Sửa task đã xong → chỉ xem</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2555,19 +2555,19 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>TASK-19</t>
+          <t>TASK-18</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Task đã xoá không còn xem được</t>
+          <t>Xoá mềm task</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2616,12 +2616,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>TASK-20</t>
+          <t>TASK-19</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Nhân viên không được xoá task</t>
+          <t>Task đã xoá không còn xem được</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2634,9 +2634,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>TASK-21</t>
+          <t>TASK-20</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager không được xoá task</t>
+          <t>Nhân viên không được xoá task</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2685,17 +2685,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>6. Milestone (Tracker)</t>
+          <t>5. Xoá task</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>MS-01</t>
+          <t>TASK-21</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo/thay toàn bộ mốc milestone lần đầu trên project</t>
+          <t>Creative Manager không được xoá task</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>MS-02</t>
+          <t>MS-01</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Sửa mốc milestone sau setup</t>
+          <t>Admin tạo/thay toàn bộ mốc milestone lần đầu trên project</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2764,12 +2764,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>MS-03</t>
+          <t>MS-02</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Thêm mốc milestone mới sau setup</t>
+          <t>Sửa mốc milestone sau setup</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2777,9 +2777,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>MS-04</t>
+          <t>MS-03</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Xóa hết mốc → project/tracker không còn mốc</t>
+          <t>Thêm mốc milestone mới sau setup</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2814,14 +2814,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>MS-05</t>
+          <t>MS-04</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>PM được ghi mốc (API 200); UI Tracker thêm mốc với seed project PM</t>
+          <t>Xóa hết mốc → project/tracker không còn mốc</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2851,14 +2851,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>MS-06</t>
+          <t>MS-05</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager được tạo mốc milestone</t>
+          <t>PM được ghi mốc (API 200); UI Tracker thêm mốc với seed project PM</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2888,9 +2888,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -2912,12 +2912,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>MS-07</t>
+          <t>MS-06</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Head được tạo mốc milestone</t>
+          <t>Creative Manager được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2925,9 +2925,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>MS-08</t>
+          <t>MS-07</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Admin được tạo mốc milestone</t>
+          <t>Head được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2986,12 +2986,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>MS-09</t>
+          <t>MS-08</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Employee không được tạo mốc; UI Tracker ẩn nút thêm/sửa mốc</t>
+          <t>Admin được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -3023,12 +3023,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>MS-10</t>
+          <t>MS-09</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Creative Head không được tạo mốc</t>
+          <t>Employee không được tạo mốc; UI Tracker ẩn nút thêm/sửa mốc</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -3036,9 +3036,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>MS-11</t>
+          <t>MS-10</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Mốc milestone không volume (unit rỗng, qty rỗng) hợp lệ; hover Tracker hiện «Tên mốc - Ghi chú»</t>
+          <t>Creative Head không được tạo mốc</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -3073,9 +3073,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>MS-12</t>
+          <t>MS-11</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>unit=slides bắt buộc quantity &gt; 0 — thiếu/≤0 → lỗi</t>
+          <t>Mốc milestone không volume (unit rỗng, qty rỗng) hợp lệ; hover Tracker hiện «Tên mốc - Ghi chú»</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -3110,9 +3110,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>MS-13</t>
+          <t>MS-12</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>unit=da bắt buộc quantity &gt; 0 — thiếu → lỗi</t>
+          <t>unit=slides bắt buộc quantity &gt; 0 — thiếu/≤0 → lỗi</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -3171,12 +3171,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>MS-14</t>
+          <t>MS-13</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Đánh dấu Hoàn thành (completed=true) → có completedAt; UI checkbox Hoàn thành trên Tracker</t>
+          <t>unit=da bắt buộc quantity &gt; 0 — thiếu → lỗi</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3184,9 +3184,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -3208,12 +3208,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>MS-15</t>
+          <t>MS-14</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Bỏ Hoàn thành (completed=false) → xóa completedAt</t>
+          <t>Đánh dấu Hoàn thành (completed=true) → có completedAt; UI checkbox Hoàn thành trên Tracker</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -3221,9 +3221,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -3245,12 +3245,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>MS-16</t>
+          <t>MS-15</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Project archived: không cho thay đổi mốc milestone</t>
+          <t>Bỏ Hoàn thành (completed=false) → xóa completedAt</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -3263,9 +3263,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F75" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>MS-17</t>
+          <t>MS-16</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Project status finish: không cho thay đổi mốc milestone</t>
+          <t>Project archived: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>MS-18</t>
+          <t>MS-17</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Project status cancel: không cho thay đổi mốc milestone</t>
+          <t>Project status finish: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>MS-19</t>
+          <t>MS-18</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>UI trên Tracker hiện chấm đỏ (#dc2626) khi chưa hoàn thành → xanh (#16a34a) khi hoàn thành</t>
+          <t>Project status cancel: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -3369,9 +3369,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>MS-20</t>
+          <t>MS-19</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Mở tracker thấy đủ mốc milestone và trạng thái màu</t>
+          <t>UI trên Tracker hiện chấm đỏ (#dc2626) khi chưa hoàn thành → xanh (#16a34a) khi hoàn thành</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -3406,14 +3406,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -3425,17 +3425,17 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>7. Tracker</t>
+          <t>6. Milestone (Tracker)</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>MS-20</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>PM đổi urgency trên Tracker (chấm ưu tiên) được; Employee bị 403</t>
+          <t>Mở tracker thấy đủ mốc milestone và trạng thái màu</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -3443,9 +3443,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>TRK-01</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>PM sửa ngày bắt đầu/kết thúc project (timeline) qua Edit Project được</t>
+          <t>PM đổi urgency trên Tracker (chấm ưu tiên) được; Employee bị 403</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -3485,9 +3485,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3504,12 +3504,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>TRK-02</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>PM/CM thêm-sửa mốc trên Tracker khớp BE (không còn FE cho / BE 403)</t>
+          <t>PM sửa ngày bắt đầu/kết thúc project (timeline) qua Edit Project được</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>TRK-04</t>
+          <t>TRK-03</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Timeline bar: deadline lịch VN 16/10 → thanh kéo hết cột 16/10 (không dừng 15/10 vì UTC)</t>
+          <t>PM/CM thêm-sửa mốc trên Tracker khớp BE (không còn FE cho / BE 403)</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -3578,30 +3578,67 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
+          <t>TRK-04</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Timeline bar: deadline lịch VN 16/10 → thanh kéo hết cột 16/10 (không dừng 15/10 vì UTC)</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>7. Tracker</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
           <t>TRK-05</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Create/Edit Project gửi start/end dạng YYYY-MM-DD (calendar VN), không toISOString lệch ngày</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G84" s="3" t="inlineStr">
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -3619,7 +3656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4086,7 +4123,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Admin: gõ tên project chưa có → Add mở Create project → tạo xong gắn tên + PM (link xanh khi tạo task)</t>
+          <t>Admin: gõ tên project chưa có → Add mở Create project (Add vẫn hiện khi không còn option khớp filter)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4137,6 +4174,38 @@
         </is>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TASK-82</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Create task: Deadline chỉ chọn ngày trong startDate–endDate của project catalog</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>●</t>
         </is>

</xml_diff>

<commit_message>
test: add TASK-85 QA child coverage and refresh workbook
Document QA add-child cases, add Playwright coverage, and sync the
task-flow Excel/checklist with TASK-83/84/85.
</commit_message>
<xml_diff>
--- a/docs/task-flow-test-cases.xlsx
+++ b/docs/task-flow-test-cases.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2167,17 +2167,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>3. Từ chối giao</t>
+          <t>2. Giao task</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>TASK-64</t>
+          <t>TASK-83</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Creative Head từ chối nhận task từ PM → task về chờ PM xử lý</t>
+          <t>Sau khi đã chia, PM thêm task con SL 0 chưa gán Staff; SL cha không đổi</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -2190,12 +2190,12 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -2204,17 +2204,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>3. Từ chối giao</t>
+          <t>2. Giao task</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>TASK-77</t>
+          <t>TASK-84</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager từ chối nhận → task về hàng chờ Creative Head</t>
+          <t>Lịch sử task cha ghi nhận chia nhỏ / thêm task con / đổi SL kèm lý do</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -2224,34 +2224,34 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>3. Từ chối giao</t>
+          <t>2. Giao task</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>TASK-78</t>
+          <t>TASK-85</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Staff từ chối task đã giao → task về Creative Manager để giao lại</t>
+          <t>PM/Admin thêm task con QA (QA 1–5); SL QA ngoài tổng cha; thiếu level / CM thêm / vượt SL phần làm → từ chối</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -2264,14 +2264,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -2283,17 +2283,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>TASK-67</t>
+          <t>TASK-64</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Nhập lý do từ chối; lịch sử / tracker ghi nhận đúng</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+          <t>Creative Head từ chối nhận task từ PM → task về chờ PM xử lý</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -2301,14 +2301,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -2320,20 +2320,20 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>TASK-79</t>
+          <t>TASK-77</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Không cho từ chối trên task cha đã chia nhỏ</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
+          <t>Creative Manager từ chối nhận → task về hàng chờ Creative Head</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -2343,26 +2343,26 @@
           <t>●</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>4. Sửa task</t>
+          <t>3. Từ chối giao</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>TASK-07–09</t>
+          <t>TASK-78</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Admin / Head / người tạo được sửa thông tin task</t>
+          <t>Staff từ chối task đã giao → task về Creative Manager để giao lại</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2370,83 +2370,83 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>~</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>4. Sửa task</t>
+          <t>3. Từ chối giao</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>TASK-10–11</t>
+          <t>TASK-67</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>PM không phải người tạo / nhân viên không được sửa meta</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+          <t>Nhập lý do từ chối; lịch sử / tracker ghi nhận đúng</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>4. Sửa task</t>
+          <t>3. Từ chối giao</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>TASK-12–13</t>
+          <t>TASK-79</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Task Hoàn thành / Hủy: không ghi được; vẫn mở xem được</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+          <t>Không cho từ chối trên task cha đã chia nhỏ</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -2454,9 +2454,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -2468,12 +2468,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>TASK-43</t>
+          <t>TASK-07–09</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Đổi mức độ ưu tiên (urgency)</t>
+          <t>Admin / Head / người tạo được sửa thông tin task</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2505,12 +2505,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>TASK-53–54</t>
+          <t>TASK-10–11</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Số lượng trước / sau khi chia nhỏ</t>
+          <t>PM không phải người tạo / nhân viên không được sửa meta</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -2523,9 +2523,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2542,12 +2542,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>TASK-68</t>
+          <t>TASK-12–13</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Staff mở task cha đã chia nhỏ → không có quyền; PM mở Sửa task đã xong → chỉ xem</t>
+          <t>Task Hoàn thành / Hủy: không ghi được; vẫn mở xem được</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2555,9 +2555,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2565,26 +2565,26 @@
           <t>●</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>5. Xoá task</t>
+          <t>4. Sửa task</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>TASK-18</t>
+          <t>TASK-43</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Xoá mềm task</t>
+          <t>Đổi mức độ ưu tiên (urgency)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2597,9 +2597,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -2611,17 +2611,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>5. Xoá task</t>
+          <t>4. Sửa task</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>TASK-19</t>
+          <t>TASK-53–54</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Task đã xoá không còn xem được</t>
+          <t>Số lượng trước / sau khi chia nhỏ</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2634,9 +2634,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2648,17 +2648,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>5. Xoá task</t>
+          <t>4. Sửa task</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>TASK-20</t>
+          <t>TASK-68</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Nhân viên không được xoá task</t>
+          <t>Staff mở task cha đã chia nhỏ → không có quyền; PM mở Sửa task đã xong → chỉ xem</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2666,19 +2666,19 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -2690,12 +2690,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>TASK-21</t>
+          <t>TASK-18</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager không được xoá task</t>
+          <t>Xoá mềm task</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2708,9 +2708,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2722,17 +2722,17 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>6. Milestone (Tracker)</t>
+          <t>5. Xoá task</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>MS-01</t>
+          <t>TASK-19</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo/thay toàn bộ mốc milestone lần đầu trên project</t>
+          <t>Task đã xoá không còn xem được</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2745,9 +2745,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2759,17 +2759,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>6. Milestone (Tracker)</t>
+          <t>5. Xoá task</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>MS-02</t>
+          <t>TASK-20</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Sửa mốc milestone sau setup</t>
+          <t>Nhân viên không được xoá task</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2796,17 +2796,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>6. Milestone (Tracker)</t>
+          <t>5. Xoá task</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>MS-03</t>
+          <t>TASK-21</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Thêm mốc milestone mới sau setup</t>
+          <t>Creative Manager không được xoá task</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2814,9 +2814,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>MS-04</t>
+          <t>MS-01</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Xóa hết mốc → project/tracker không còn mốc</t>
+          <t>Admin tạo/thay toàn bộ mốc milestone lần đầu trên project</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2856,9 +2856,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>MS-05</t>
+          <t>MS-02</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>PM được ghi mốc (API 200); UI Tracker thêm mốc với seed project PM</t>
+          <t>Sửa mốc milestone sau setup</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2888,14 +2888,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -2912,12 +2912,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>MS-06</t>
+          <t>MS-03</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Creative Manager được tạo mốc milestone</t>
+          <t>Thêm mốc milestone mới sau setup</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2925,14 +2925,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>MS-07</t>
+          <t>MS-04</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Head được tạo mốc milestone</t>
+          <t>Xóa hết mốc → project/tracker không còn mốc</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2962,14 +2962,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -2986,12 +2986,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>MS-08</t>
+          <t>MS-05</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Admin được tạo mốc milestone</t>
+          <t>PM được ghi mốc (API 200); UI Tracker thêm mốc với seed project PM</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -3023,12 +3023,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>MS-09</t>
+          <t>MS-06</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Employee không được tạo mốc; UI Tracker ẩn nút thêm/sửa mốc</t>
+          <t>Creative Manager được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -3036,9 +3036,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>MS-10</t>
+          <t>MS-07</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Creative Head không được tạo mốc</t>
+          <t>Head được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -3073,9 +3073,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>MS-11</t>
+          <t>MS-08</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Mốc milestone không volume (unit rỗng, qty rỗng) hợp lệ; hover Tracker hiện «Tên mốc - Ghi chú»</t>
+          <t>Admin được tạo mốc milestone</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>MS-12</t>
+          <t>MS-09</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>unit=slides bắt buộc quantity &gt; 0 — thiếu/≤0 → lỗi</t>
+          <t>Employee không được tạo mốc; UI Tracker ẩn nút thêm/sửa mốc</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -3147,9 +3147,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -3171,12 +3171,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>MS-13</t>
+          <t>MS-10</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>unit=da bắt buộc quantity &gt; 0 — thiếu → lỗi</t>
+          <t>Creative Head không được tạo mốc</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3208,12 +3208,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>MS-14</t>
+          <t>MS-11</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Đánh dấu Hoàn thành (completed=true) → có completedAt; UI checkbox Hoàn thành trên Tracker</t>
+          <t>Mốc milestone không volume (unit rỗng, qty rỗng) hợp lệ; hover Tracker hiện «Tên mốc - Ghi chú»</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -3245,12 +3245,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>MS-15</t>
+          <t>MS-12</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Bỏ Hoàn thành (completed=false) → xóa completedAt</t>
+          <t>unit=slides bắt buộc quantity &gt; 0 — thiếu/≤0 → lỗi</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>MS-16</t>
+          <t>MS-13</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Project archived: không cho thay đổi mốc milestone</t>
+          <t>unit=da bắt buộc quantity &gt; 0 — thiếu → lỗi</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -3300,9 +3300,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F76" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>MS-17</t>
+          <t>MS-14</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Project status finish: không cho thay đổi mốc milestone</t>
+          <t>Đánh dấu Hoàn thành (completed=true) → có completedAt; UI checkbox Hoàn thành trên Tracker</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -3332,14 +3332,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="F77" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>MS-18</t>
+          <t>MS-15</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Project status cancel: không cho thay đổi mốc milestone</t>
+          <t>Bỏ Hoàn thành (completed=false) → xóa completedAt</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -3374,9 +3374,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F78" s="5" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>MS-19</t>
+          <t>MS-16</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>UI trên Tracker hiện chấm đỏ (#dc2626) khi chưa hoàn thành → xanh (#16a34a) khi hoàn thành</t>
+          <t>Project archived: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -3406,9 +3406,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -3430,12 +3430,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>MS-20</t>
+          <t>MS-17</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Mở tracker thấy đủ mốc milestone và trạng thái màu</t>
+          <t>Project status finish: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -3448,9 +3448,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3462,17 +3462,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>7. Tracker</t>
+          <t>6. Milestone (Tracker)</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>MS-18</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>PM đổi urgency trên Tracker (chấm ưu tiên) được; Employee bị 403</t>
+          <t>Project status cancel: không cho thay đổi mốc milestone</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -3480,14 +3480,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3499,17 +3499,17 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>7. Tracker</t>
+          <t>6. Milestone (Tracker)</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>MS-19</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>PM sửa ngày bắt đầu/kết thúc project (timeline) qua Edit Project được</t>
+          <t>UI trên Tracker hiện chấm đỏ (#dc2626) khi chưa hoàn thành → xanh (#16a34a) khi hoàn thành</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -3522,9 +3522,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -3536,17 +3536,17 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>7. Tracker</t>
+          <t>6. Milestone (Tracker)</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>MS-20</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>PM/CM thêm-sửa mốc trên Tracker khớp BE (không còn FE cho / BE 403)</t>
+          <t>Mở tracker thấy đủ mốc milestone và trạng thái màu</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -3554,14 +3554,14 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -3578,12 +3578,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>TRK-04</t>
+          <t>TRK-01</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Timeline bar: deadline lịch VN 16/10 → thanh kéo hết cột 16/10 (không dừng 15/10 vì UTC)</t>
+          <t>PM đổi urgency trên Tracker (chấm ưu tiên) được; Employee bị 403</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -3596,9 +3596,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3615,30 +3615,141 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>TRK-02</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>PM sửa ngày bắt đầu/kết thúc project (timeline) qua Edit Project được</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>7. Tracker</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>TRK-03</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>PM/CM thêm-sửa mốc trên Tracker khớp BE (không còn FE cho / BE 403)</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>7. Tracker</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>TRK-04</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Timeline bar: deadline lịch VN 16/10 → thanh kéo hết cột 16/10 (không dừng 15/10 vì UTC)</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>7. Tracker</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>TRK-05</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Create/Edit Project gửi start/end dạng YYYY-MM-DD (calendar VN), không toISOString lệch ngày</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="inlineStr">
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -4223,7 +4334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5159,6 +5270,102 @@
       <c r="F29" s="4" t="inlineStr">
         <is>
           <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TASK-83</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Sau khi đã chia, PM thêm task con SL 0 chưa gán Staff; SL cha không đổi</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TASK-84</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử task cha ghi nhận chia nhỏ / thêm task con / đổi SL kèm lý do</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TASK-85</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>PM/Admin thêm task con QA (QA 1–5); SL QA ngoài tổng cha; thiếu level / CM thêm / vượt SL phần làm → từ chối</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>●</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6976,6 +7183,42 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TASK-83</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>PM thêm task con SL 0 · e2e/tasks/task-83-… · API TASK83</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TASK-84</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Audit history chia/thêm con/đổi SL · API TASK84</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TASK-85</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Task con QA ngoài SL tổng · e2e/tasks/task-85-… · API TASK85 · mock unit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>